<commit_message>
Adding the largest batch of files since Jan '26 slx files have been edited and added which contribute to the major issues here: - libs_unified.slx has be altered to appeal to the correct sensing   algorithm for milliseconds parameterisation - CLSfixed now includes various tests for different output methods - CLSfixed_nopace outputs EGMs which can then be passed into a function   generator - CLSfixed_pace includes simulated communication delays between the code - myocyteM/myocyteNM/pacemakerN slx files are different restitution   curve computation models which currently do not work to expectation - HeartGUI[_preset] are updated but are pseudo-deprecated - Major changes done with the editing app which now includes reading in   CellML action potential traces and limited probe editing   functionality.
</commit_message>
<xml_diff>
--- a/src/Heart_N3_second.xlsx
+++ b/src/Heart_N3_second.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3B5180F-8CF3-44C1-989E-F6C4CF040466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24F52071-9DA1-45D7-917C-7739A5CFB14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Node_second" sheetId="39" r:id="rId1"/>
@@ -30,6 +30,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Node_second!$A:$C</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>